<commit_message>
TwoWaySQL	v2.7.0 Added support for MxDBUnit's external DB testing functionality. Added the GetOrderByFromGridState action.
TwoWaySQLMocker		v1.0.2
Fixed an issue where date/time fields in Excel mock data lacking a specified time zone were not being read using the session or default time zone.
</commit_message>
<xml_diff>
--- a/src/MxTwoWaySql/resources/sql/mockdata/test1.xlsx
+++ b/src/MxTwoWaySql/resources/sql/mockdata/test1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\tmp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\MxTwoWaySql\src\MxTwoWaySql\resources\sql\mockdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA19EA1C-C80D-4D9D-8210-58E7F039EBAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{234A8877-83EC-44C2-BAAE-0488B330BF78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="50172" yWindow="300" windowWidth="18468" windowHeight="12120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="54156" yWindow="948" windowWidth="14820" windowHeight="10740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>田中</t>
     <rPh sb="0" eb="2">
@@ -93,13 +93,6 @@
     <phoneticPr fontId="1"/>
   </si>
   <si>
-    <t>埼玉</t>
-    <rPh sb="0" eb="2">
-      <t>サイタマ</t>
-    </rPh>
-    <phoneticPr fontId="1"/>
-  </si>
-  <si>
     <t>IsHoge</t>
     <phoneticPr fontId="1"/>
   </si>
@@ -109,6 +102,17 @@
   </si>
   <si>
     <t>IntVal</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>1964-01-13T00:00:00</t>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>茨城</t>
+    <rPh sb="0" eb="2">
+      <t>イバラキ</t>
+    </rPh>
     <phoneticPr fontId="1"/>
   </si>
 </sst>
@@ -458,13 +462,13 @@
         <v>8</v>
       </c>
       <c r="E1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1" t="s">
         <v>13</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>14</v>
-      </c>
-      <c r="G1" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.45">
@@ -527,10 +531,13 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="C5" t="s">
-        <v>12</v>
+        <v>16</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
       </c>
       <c r="E5" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
We have improved XssfExcelReader so that it skips empty rows.
</commit_message>
<xml_diff>
--- a/src/MxTwoWaySql/resources/sql/mockdata/test1.xlsx
+++ b/src/MxTwoWaySql/resources/sql/mockdata/test1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\MxTwoWaySql\src\MxTwoWaySql\resources\sql\mockdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{234A8877-83EC-44C2-BAAE-0488B330BF78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0E88A25-4704-4E8F-97EC-90CE376E0B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="54156" yWindow="948" windowWidth="14820" windowHeight="10740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28920" yWindow="-6300" windowWidth="34560" windowHeight="18600" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -442,7 +442,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="4" max="4" width="26.19921875" bestFit="1" customWidth="1"/>
@@ -514,35 +514,35 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" s="1"/>
-      <c r="E4" t="b">
-        <v>0</v>
-      </c>
-      <c r="G4">
-        <v>3</v>
-      </c>
-    </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="1"/>
+      <c r="E5" t="b">
+        <v>0</v>
+      </c>
+      <c r="G5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
         <v>4</v>
       </c>
-      <c r="B5">
+      <c r="B6">
         <v>62</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C6" t="s">
         <v>16</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D6" t="s">
         <v>15</v>
       </c>
-      <c r="E5" t="b">
+      <c r="E6" t="b">
         <v>1</v>
       </c>
-      <c r="F5">
+      <c r="F6">
         <v>999.99</v>
       </c>
     </row>

</xml_diff>